<commit_message>
Remove evaluation language from candidate task
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R3d7059dab8f74b0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R7fe6f192e2924946"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -540,7 +540,7 @@
         <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
-        <x:v>npm run compile:push返回0，五个目标路径可读，四份报告以template_id、locale和job_id闭合</x:v>
+        <x:v>npm run compile:push返回0，Prompt声明的目标路径可读，业务报告以template_id、locale和job_id闭合</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">

</xml_diff>